<commit_message>
Bulk-update Shopify unit costs from CJ master sheet (182 variants verified), refresh cost table and verification workbook
</commit_message>
<xml_diff>
--- a/data/product-costs-2026-07-22.xlsx
+++ b/data/product-costs-2026-07-22.xlsx
@@ -501,7 +501,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時: 2026-07-22 定例後（更新前ベースライン）。F列=現在Shopifyに登録されている原価。G列（黄色）に新しい原価を記入してください（円・整数・送料込み。例: 1234）。変更のない行は空欄のままでOK。</t>
+          <t>2026-07-22 原価一括更新の検証記録。E列=更新前 / F列=新原価(Google原価表I列) / G列=Shopify再取得の実測照合結果。全ACTIVE 182バリエーション更新・全行一致を確認済み。非ACTIVE商品はユーザー指示により対象外。形状記憶日傘は完全遮光UV日傘と同一SPU(CJYD2824705)のため同額1309円を適用。ナノガラスは白/緑757・黒/ピンク740の色別。</t>
         </is>
       </c>
     </row>
@@ -564,8 +564,14 @@
       <c r="E5" s="5" t="n">
         <v>2484</v>
       </c>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="4" t="inlineStr"/>
+      <c r="F5" s="6" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2484→2500</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -589,8 +595,14 @@
       <c r="E6" s="5" t="n">
         <v>2484</v>
       </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="4" t="inlineStr"/>
+      <c r="F6" s="6" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2484→2500</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -614,8 +626,14 @@
       <c r="E7" s="5" t="n">
         <v>2484</v>
       </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="4" t="inlineStr"/>
+      <c r="F7" s="6" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2484→2500</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -639,8 +657,14 @@
       <c r="E8" s="5" t="n">
         <v>2484</v>
       </c>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="4" t="inlineStr"/>
+      <c r="F8" s="6" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2484→2500</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -664,8 +688,14 @@
       <c r="E9" s="5" t="n">
         <v>1708</v>
       </c>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="4" t="inlineStr"/>
+      <c r="F9" s="6" t="n">
+        <v>1730</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1708→1730</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -689,8 +719,14 @@
       <c r="E10" s="5" t="n">
         <v>1708</v>
       </c>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="4" t="inlineStr"/>
+      <c r="F10" s="6" t="n">
+        <v>1730</v>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1708→1730</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -714,8 +750,14 @@
       <c r="E11" s="5" t="n">
         <v>1708</v>
       </c>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="4" t="inlineStr"/>
+      <c r="F11" s="6" t="n">
+        <v>1730</v>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1708→1730</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -739,8 +781,14 @@
       <c r="E12" s="5" t="n">
         <v>1708</v>
       </c>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="4" t="inlineStr"/>
+      <c r="F12" s="6" t="n">
+        <v>1730</v>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1708→1730</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -764,8 +812,14 @@
       <c r="E13" s="5" t="n">
         <v>1853</v>
       </c>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="4" t="inlineStr"/>
+      <c r="F13" s="6" t="n">
+        <v>1848</v>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1853→1848</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -789,8 +843,14 @@
       <c r="E14" s="5" t="n">
         <v>1853</v>
       </c>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="4" t="inlineStr"/>
+      <c r="F14" s="6" t="n">
+        <v>1848</v>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1853→1848</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -814,8 +874,14 @@
       <c r="E15" s="5" t="n">
         <v>3605</v>
       </c>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="4" t="inlineStr"/>
+      <c r="F15" s="6" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  3605→3480</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -839,8 +905,14 @@
       <c r="E16" s="5" t="n">
         <v>3605</v>
       </c>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="4" t="inlineStr"/>
+      <c r="F16" s="6" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  3605→3480</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -864,8 +936,14 @@
       <c r="E17" s="5" t="n">
         <v>3269</v>
       </c>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="4" t="inlineStr"/>
+      <c r="F17" s="6" t="n">
+        <v>3191</v>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  3269→3191</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -889,8 +967,14 @@
       <c r="E18" s="5" t="n">
         <v>1612</v>
       </c>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="4" t="inlineStr"/>
+      <c r="F18" s="6" t="n">
+        <v>1398</v>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1612→1398</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -914,8 +998,14 @@
       <c r="E19" s="5" t="n">
         <v>1612</v>
       </c>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="4" t="inlineStr"/>
+      <c r="F19" s="6" t="n">
+        <v>1398</v>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1612→1398</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -939,8 +1029,14 @@
       <c r="E20" s="5" t="n">
         <v>1612</v>
       </c>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="4" t="inlineStr"/>
+      <c r="F20" s="6" t="n">
+        <v>1398</v>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1612→1398</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -964,8 +1060,14 @@
       <c r="E21" s="5" t="n">
         <v>1578</v>
       </c>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="4" t="inlineStr"/>
+      <c r="F21" s="6" t="n">
+        <v>1213</v>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1578→1213</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -989,8 +1091,14 @@
       <c r="E22" s="5" t="n">
         <v>1578</v>
       </c>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="4" t="inlineStr"/>
+      <c r="F22" s="6" t="n">
+        <v>1213</v>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1578→1213</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -1014,8 +1122,14 @@
       <c r="E23" s="5" t="n">
         <v>1578</v>
       </c>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="4" t="inlineStr"/>
+      <c r="F23" s="6" t="n">
+        <v>1213</v>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1578→1213</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -1039,8 +1153,14 @@
       <c r="E24" s="5" t="n">
         <v>1578</v>
       </c>
-      <c r="F24" s="6" t="n"/>
-      <c r="G24" s="4" t="inlineStr"/>
+      <c r="F24" s="6" t="n">
+        <v>1213</v>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1578→1213</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -1064,8 +1184,14 @@
       <c r="E25" s="5" t="n">
         <v>1578</v>
       </c>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="4" t="inlineStr"/>
+      <c r="F25" s="6" t="n">
+        <v>1213</v>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1578→1213</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -1089,8 +1215,14 @@
       <c r="E26" s="5" t="n">
         <v>1578</v>
       </c>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="4" t="inlineStr"/>
+      <c r="F26" s="6" t="n">
+        <v>1213</v>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1578→1213</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -1114,8 +1246,14 @@
       <c r="E27" s="5" t="n">
         <v>1578</v>
       </c>
-      <c r="F27" s="6" t="n"/>
-      <c r="G27" s="4" t="inlineStr"/>
+      <c r="F27" s="6" t="n">
+        <v>1213</v>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1578→1213</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -1139,8 +1277,14 @@
       <c r="E28" s="5" t="n">
         <v>1578</v>
       </c>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" s="4" t="inlineStr"/>
+      <c r="F28" s="6" t="n">
+        <v>1213</v>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1578→1213</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -1164,8 +1308,14 @@
       <c r="E29" s="5" t="n">
         <v>2489</v>
       </c>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" s="4" t="inlineStr"/>
+      <c r="F29" s="6" t="n">
+        <v>2453</v>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2489→2453</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -1189,8 +1339,14 @@
       <c r="E30" s="5" t="n">
         <v>747</v>
       </c>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="4" t="inlineStr"/>
+      <c r="F30" s="6" t="n">
+        <v>757</v>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  747→757</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -1214,8 +1370,14 @@
       <c r="E31" s="5" t="n">
         <v>747</v>
       </c>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="4" t="inlineStr"/>
+      <c r="F31" s="6" t="n">
+        <v>740</v>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  747→740</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -1239,8 +1401,14 @@
       <c r="E32" s="5" t="n">
         <v>747</v>
       </c>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="4" t="inlineStr"/>
+      <c r="F32" s="6" t="n">
+        <v>757</v>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  747→757</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -1264,8 +1432,14 @@
       <c r="E33" s="5" t="n">
         <v>747</v>
       </c>
-      <c r="F33" s="6" t="n"/>
-      <c r="G33" s="4" t="inlineStr"/>
+      <c r="F33" s="6" t="n">
+        <v>740</v>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  747→740</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -1289,8 +1463,14 @@
       <c r="E34" s="5" t="n">
         <v>2636</v>
       </c>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="4" t="inlineStr"/>
+      <c r="F34" s="6" t="n">
+        <v>2333</v>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2636→2333</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -1314,8 +1494,14 @@
       <c r="E35" s="5" t="n">
         <v>5553</v>
       </c>
-      <c r="F35" s="6" t="n"/>
-      <c r="G35" s="4" t="inlineStr"/>
+      <c r="F35" s="6" t="n">
+        <v>3136</v>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  5553→3136</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -1339,8 +1525,14 @@
       <c r="E36" s="5" t="n">
         <v>1288</v>
       </c>
-      <c r="F36" s="6" t="n"/>
-      <c r="G36" s="4" t="inlineStr"/>
+      <c r="F36" s="6" t="n">
+        <v>1304</v>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1288→1304</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -1364,8 +1556,14 @@
       <c r="E37" s="5" t="n">
         <v>1288</v>
       </c>
-      <c r="F37" s="6" t="n"/>
-      <c r="G37" s="4" t="inlineStr"/>
+      <c r="F37" s="6" t="n">
+        <v>1304</v>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1288→1304</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -1389,8 +1587,14 @@
       <c r="E38" s="5" t="n">
         <v>1288</v>
       </c>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="4" t="inlineStr"/>
+      <c r="F38" s="6" t="n">
+        <v>1304</v>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1288→1304</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -1414,8 +1618,14 @@
       <c r="E39" s="5" t="n">
         <v>1288</v>
       </c>
-      <c r="F39" s="6" t="n"/>
-      <c r="G39" s="4" t="inlineStr"/>
+      <c r="F39" s="6" t="n">
+        <v>1304</v>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1288→1304</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -1439,8 +1649,14 @@
       <c r="E40" s="5" t="n">
         <v>2800</v>
       </c>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" s="4" t="inlineStr"/>
+      <c r="F40" s="6" t="n">
+        <v>2798</v>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2800→2798</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -1464,8 +1680,14 @@
       <c r="E41" s="5" t="n">
         <v>2800</v>
       </c>
-      <c r="F41" s="6" t="n"/>
-      <c r="G41" s="4" t="inlineStr"/>
+      <c r="F41" s="6" t="n">
+        <v>2798</v>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2800→2798</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
@@ -1489,8 +1711,14 @@
       <c r="E42" s="5" t="n">
         <v>2800</v>
       </c>
-      <c r="F42" s="6" t="n"/>
-      <c r="G42" s="4" t="inlineStr"/>
+      <c r="F42" s="6" t="n">
+        <v>2798</v>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2800→2798</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -1514,8 +1742,14 @@
       <c r="E43" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F43" s="6" t="n"/>
-      <c r="G43" s="4" t="inlineStr"/>
+      <c r="F43" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
@@ -1539,8 +1773,14 @@
       <c r="E44" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F44" s="6" t="n"/>
-      <c r="G44" s="4" t="inlineStr"/>
+      <c r="F44" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -1564,8 +1804,14 @@
       <c r="E45" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F45" s="6" t="n"/>
-      <c r="G45" s="4" t="inlineStr"/>
+      <c r="F45" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
@@ -1589,8 +1835,14 @@
       <c r="E46" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F46" s="6" t="n"/>
-      <c r="G46" s="4" t="inlineStr"/>
+      <c r="F46" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -1614,8 +1866,14 @@
       <c r="E47" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F47" s="6" t="n"/>
-      <c r="G47" s="4" t="inlineStr"/>
+      <c r="F47" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
@@ -1639,8 +1897,14 @@
       <c r="E48" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F48" s="6" t="n"/>
-      <c r="G48" s="4" t="inlineStr"/>
+      <c r="F48" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -1664,8 +1928,14 @@
       <c r="E49" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F49" s="6" t="n"/>
-      <c r="G49" s="4" t="inlineStr"/>
+      <c r="F49" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n">
@@ -1689,8 +1959,14 @@
       <c r="E50" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F50" s="6" t="n"/>
-      <c r="G50" s="4" t="inlineStr"/>
+      <c r="F50" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -1714,8 +1990,14 @@
       <c r="E51" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F51" s="6" t="n"/>
-      <c r="G51" s="4" t="inlineStr"/>
+      <c r="F51" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
@@ -1739,8 +2021,14 @@
       <c r="E52" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F52" s="6" t="n"/>
-      <c r="G52" s="4" t="inlineStr"/>
+      <c r="F52" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -1764,8 +2052,14 @@
       <c r="E53" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F53" s="6" t="n"/>
-      <c r="G53" s="4" t="inlineStr"/>
+      <c r="F53" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -1789,8 +2083,14 @@
       <c r="E54" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F54" s="6" t="n"/>
-      <c r="G54" s="4" t="inlineStr"/>
+      <c r="F54" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
@@ -1814,8 +2114,14 @@
       <c r="E55" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F55" s="6" t="n"/>
-      <c r="G55" s="4" t="inlineStr"/>
+      <c r="F55" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n">
@@ -1839,8 +2145,14 @@
       <c r="E56" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F56" s="6" t="n"/>
-      <c r="G56" s="4" t="inlineStr"/>
+      <c r="F56" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -1864,8 +2176,14 @@
       <c r="E57" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F57" s="6" t="n"/>
-      <c r="G57" s="4" t="inlineStr"/>
+      <c r="F57" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n">
@@ -1889,8 +2207,14 @@
       <c r="E58" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F58" s="6" t="n"/>
-      <c r="G58" s="4" t="inlineStr"/>
+      <c r="F58" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n">
@@ -1914,8 +2238,14 @@
       <c r="E59" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F59" s="6" t="n"/>
-      <c r="G59" s="4" t="inlineStr"/>
+      <c r="F59" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n">
@@ -1939,8 +2269,14 @@
       <c r="E60" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F60" s="6" t="n"/>
-      <c r="G60" s="4" t="inlineStr"/>
+      <c r="F60" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n">
@@ -1964,8 +2300,14 @@
       <c r="E61" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F61" s="6" t="n"/>
-      <c r="G61" s="4" t="inlineStr"/>
+      <c r="F61" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="n">
@@ -1989,8 +2331,14 @@
       <c r="E62" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F62" s="6" t="n"/>
-      <c r="G62" s="4" t="inlineStr"/>
+      <c r="F62" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n">
@@ -2014,8 +2362,14 @@
       <c r="E63" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F63" s="6" t="n"/>
-      <c r="G63" s="4" t="inlineStr"/>
+      <c r="F63" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n">
@@ -2039,8 +2393,14 @@
       <c r="E64" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F64" s="6" t="n"/>
-      <c r="G64" s="4" t="inlineStr"/>
+      <c r="F64" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n">
@@ -2064,8 +2424,14 @@
       <c r="E65" s="5" t="n">
         <v>1484</v>
       </c>
-      <c r="F65" s="6" t="n"/>
-      <c r="G65" s="4" t="inlineStr"/>
+      <c r="F65" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1484→1375</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n">
@@ -2089,8 +2455,14 @@
       <c r="E66" s="5" t="n">
         <v>3952</v>
       </c>
-      <c r="F66" s="6" t="n"/>
-      <c r="G66" s="4" t="inlineStr"/>
+      <c r="F66" s="6" t="n">
+        <v>3886</v>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  3952→3886</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n">
@@ -2114,8 +2486,14 @@
       <c r="E67" s="5" t="n">
         <v>964</v>
       </c>
-      <c r="F67" s="6" t="n"/>
-      <c r="G67" s="4" t="inlineStr"/>
+      <c r="F67" s="6" t="n">
+        <v>977</v>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  964→977</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="n">
@@ -2139,8 +2517,14 @@
       <c r="E68" s="5" t="n">
         <v>964</v>
       </c>
-      <c r="F68" s="6" t="n"/>
-      <c r="G68" s="4" t="inlineStr"/>
+      <c r="F68" s="6" t="n">
+        <v>977</v>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  964→977</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n">
@@ -2164,8 +2548,14 @@
       <c r="E69" s="5" t="n">
         <v>964</v>
       </c>
-      <c r="F69" s="6" t="n"/>
-      <c r="G69" s="4" t="inlineStr"/>
+      <c r="F69" s="6" t="n">
+        <v>977</v>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  964→977</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n">
@@ -2189,8 +2579,14 @@
       <c r="E70" s="5" t="n">
         <v>964</v>
       </c>
-      <c r="F70" s="6" t="n"/>
-      <c r="G70" s="4" t="inlineStr"/>
+      <c r="F70" s="6" t="n">
+        <v>977</v>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  964→977</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n">
@@ -2214,8 +2610,14 @@
       <c r="E71" s="5" t="n">
         <v>964</v>
       </c>
-      <c r="F71" s="6" t="n"/>
-      <c r="G71" s="4" t="inlineStr"/>
+      <c r="F71" s="6" t="n">
+        <v>977</v>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  964→977</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="n">
@@ -2239,8 +2641,14 @@
       <c r="E72" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F72" s="6" t="n"/>
-      <c r="G72" s="4" t="inlineStr"/>
+      <c r="F72" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n">
@@ -2264,8 +2672,14 @@
       <c r="E73" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F73" s="6" t="n"/>
-      <c r="G73" s="4" t="inlineStr"/>
+      <c r="F73" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n">
@@ -2289,8 +2703,14 @@
       <c r="E74" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F74" s="6" t="n"/>
-      <c r="G74" s="4" t="inlineStr"/>
+      <c r="F74" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n">
@@ -2314,8 +2734,14 @@
       <c r="E75" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F75" s="6" t="n"/>
-      <c r="G75" s="4" t="inlineStr"/>
+      <c r="F75" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="n">
@@ -2339,8 +2765,14 @@
       <c r="E76" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F76" s="6" t="n"/>
-      <c r="G76" s="4" t="inlineStr"/>
+      <c r="F76" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
@@ -2364,8 +2796,14 @@
       <c r="E77" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F77" s="6" t="n"/>
-      <c r="G77" s="4" t="inlineStr"/>
+      <c r="F77" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n">
@@ -2389,8 +2827,14 @@
       <c r="E78" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F78" s="6" t="n"/>
-      <c r="G78" s="4" t="inlineStr"/>
+      <c r="F78" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n">
@@ -2414,8 +2858,14 @@
       <c r="E79" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F79" s="6" t="n"/>
-      <c r="G79" s="4" t="inlineStr"/>
+      <c r="F79" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="n">
@@ -2439,8 +2889,14 @@
       <c r="E80" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F80" s="6" t="n"/>
-      <c r="G80" s="4" t="inlineStr"/>
+      <c r="F80" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n">
@@ -2464,8 +2920,14 @@
       <c r="E81" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F81" s="6" t="n"/>
-      <c r="G81" s="4" t="inlineStr"/>
+      <c r="F81" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n">
@@ -2489,8 +2951,14 @@
       <c r="E82" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F82" s="6" t="n"/>
-      <c r="G82" s="4" t="inlineStr"/>
+      <c r="F82" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n">
@@ -2514,8 +2982,14 @@
       <c r="E83" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F83" s="6" t="n"/>
-      <c r="G83" s="4" t="inlineStr"/>
+      <c r="F83" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="n">
@@ -2539,8 +3013,14 @@
       <c r="E84" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F84" s="6" t="n"/>
-      <c r="G84" s="4" t="inlineStr"/>
+      <c r="F84" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -2564,8 +3044,14 @@
       <c r="E85" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F85" s="6" t="n"/>
-      <c r="G85" s="4" t="inlineStr"/>
+      <c r="F85" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="n">
@@ -2589,8 +3075,14 @@
       <c r="E86" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F86" s="6" t="n"/>
-      <c r="G86" s="4" t="inlineStr"/>
+      <c r="F86" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
@@ -2614,8 +3106,14 @@
       <c r="E87" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F87" s="6" t="n"/>
-      <c r="G87" s="4" t="inlineStr"/>
+      <c r="F87" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="n">
@@ -2639,8 +3137,14 @@
       <c r="E88" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F88" s="6" t="n"/>
-      <c r="G88" s="4" t="inlineStr"/>
+      <c r="F88" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
@@ -2664,8 +3168,14 @@
       <c r="E89" s="5" t="n">
         <v>1208</v>
       </c>
-      <c r="F89" s="6" t="n"/>
-      <c r="G89" s="4" t="inlineStr"/>
+      <c r="F89" s="6" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1208→1262</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="n">
@@ -2690,7 +3200,7 @@
       <c r="F90" s="6" t="n"/>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>原価未登録</t>
+          <t>原価未登録 原価対象外</t>
         </is>
       </c>
     </row>
@@ -2716,8 +3226,14 @@
       <c r="E91" s="5" t="n">
         <v>1971</v>
       </c>
-      <c r="F91" s="6" t="n"/>
-      <c r="G91" s="4" t="inlineStr"/>
+      <c r="F91" s="6" t="n">
+        <v>1996</v>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1971→1996</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="n">
@@ -2741,8 +3257,14 @@
       <c r="E92" s="5" t="n">
         <v>2441</v>
       </c>
-      <c r="F92" s="6" t="n"/>
-      <c r="G92" s="4" t="inlineStr"/>
+      <c r="F92" s="6" t="n">
+        <v>2621</v>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2441→2621</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n">
@@ -2766,8 +3288,14 @@
       <c r="E93" s="5" t="n">
         <v>2441</v>
       </c>
-      <c r="F93" s="6" t="n"/>
-      <c r="G93" s="4" t="inlineStr"/>
+      <c r="F93" s="6" t="n">
+        <v>2621</v>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2441→2621</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="n">
@@ -2791,8 +3319,14 @@
       <c r="E94" s="5" t="n">
         <v>2441</v>
       </c>
-      <c r="F94" s="6" t="n"/>
-      <c r="G94" s="4" t="inlineStr"/>
+      <c r="F94" s="6" t="n">
+        <v>2621</v>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2441→2621</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n">
@@ -2816,8 +3350,14 @@
       <c r="E95" s="5" t="n">
         <v>2441</v>
       </c>
-      <c r="F95" s="6" t="n"/>
-      <c r="G95" s="4" t="inlineStr"/>
+      <c r="F95" s="6" t="n">
+        <v>2621</v>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2441→2621</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="n">
@@ -2841,8 +3381,14 @@
       <c r="E96" s="5" t="n">
         <v>1932</v>
       </c>
-      <c r="F96" s="6" t="n"/>
-      <c r="G96" s="4" t="inlineStr"/>
+      <c r="F96" s="6" t="n">
+        <v>1981</v>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1932→1981</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="n">
@@ -2866,8 +3412,14 @@
       <c r="E97" s="5" t="n">
         <v>1932</v>
       </c>
-      <c r="F97" s="6" t="n"/>
-      <c r="G97" s="4" t="inlineStr"/>
+      <c r="F97" s="6" t="n">
+        <v>1981</v>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1932→1981</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="n">
@@ -2891,8 +3443,14 @@
       <c r="E98" s="5" t="n">
         <v>1932</v>
       </c>
-      <c r="F98" s="6" t="n"/>
-      <c r="G98" s="4" t="inlineStr"/>
+      <c r="F98" s="6" t="n">
+        <v>1981</v>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1932→1981</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n">
@@ -2916,8 +3474,14 @@
       <c r="E99" s="5" t="n">
         <v>1932</v>
       </c>
-      <c r="F99" s="6" t="n"/>
-      <c r="G99" s="4" t="inlineStr"/>
+      <c r="F99" s="6" t="n">
+        <v>1981</v>
+      </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1932→1981</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="n">
@@ -2941,8 +3505,14 @@
       <c r="E100" s="5" t="n">
         <v>4103</v>
       </c>
-      <c r="F100" s="6" t="n"/>
-      <c r="G100" s="4" t="inlineStr"/>
+      <c r="F100" s="6" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  4103→1905</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="n">
@@ -2966,8 +3536,14 @@
       <c r="E101" s="5" t="n">
         <v>4103</v>
       </c>
-      <c r="F101" s="6" t="n"/>
-      <c r="G101" s="4" t="inlineStr"/>
+      <c r="F101" s="6" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  4103→1905</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="n">
@@ -2991,8 +3567,14 @@
       <c r="E102" s="5" t="n">
         <v>4103</v>
       </c>
-      <c r="F102" s="6" t="n"/>
-      <c r="G102" s="4" t="inlineStr"/>
+      <c r="F102" s="6" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  4103→1905</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="n">
@@ -3016,8 +3598,14 @@
       <c r="E103" s="5" t="n">
         <v>4103</v>
       </c>
-      <c r="F103" s="6" t="n"/>
-      <c r="G103" s="4" t="inlineStr"/>
+      <c r="F103" s="6" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  4103→1905</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="n">
@@ -3041,8 +3629,14 @@
       <c r="E104" s="5" t="n">
         <v>1491</v>
       </c>
-      <c r="F104" s="6" t="n"/>
-      <c r="G104" s="4" t="inlineStr"/>
+      <c r="F104" s="6" t="n">
+        <v>1429</v>
+      </c>
+      <c r="G104" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1491→1429</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="n">
@@ -3066,8 +3660,14 @@
       <c r="E105" s="5" t="n">
         <v>1509</v>
       </c>
-      <c r="F105" s="6" t="n"/>
-      <c r="G105" s="4" t="inlineStr"/>
+      <c r="F105" s="6" t="n">
+        <v>1429</v>
+      </c>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1509→1429</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="4" t="n">
@@ -3091,8 +3691,14 @@
       <c r="E106" s="5" t="n">
         <v>1530</v>
       </c>
-      <c r="F106" s="6" t="n"/>
-      <c r="G106" s="4" t="inlineStr"/>
+      <c r="F106" s="6" t="n">
+        <v>1429</v>
+      </c>
+      <c r="G106" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1530→1429</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="n">
@@ -3116,8 +3722,14 @@
       <c r="E107" s="5" t="n">
         <v>1518</v>
       </c>
-      <c r="F107" s="6" t="n"/>
-      <c r="G107" s="4" t="inlineStr"/>
+      <c r="F107" s="6" t="n">
+        <v>1456</v>
+      </c>
+      <c r="G107" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1518→1456</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="n">
@@ -3141,8 +3753,14 @@
       <c r="E108" s="5" t="n">
         <v>1536</v>
       </c>
-      <c r="F108" s="6" t="n"/>
-      <c r="G108" s="4" t="inlineStr"/>
+      <c r="F108" s="6" t="n">
+        <v>1456</v>
+      </c>
+      <c r="G108" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1536→1456</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="n">
@@ -3166,8 +3784,14 @@
       <c r="E109" s="5" t="n">
         <v>1557</v>
       </c>
-      <c r="F109" s="6" t="n"/>
-      <c r="G109" s="4" t="inlineStr"/>
+      <c r="F109" s="6" t="n">
+        <v>1456</v>
+      </c>
+      <c r="G109" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1557→1456</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="n">
@@ -3191,8 +3815,14 @@
       <c r="E110" s="5" t="n">
         <v>1292</v>
       </c>
-      <c r="F110" s="6" t="n"/>
-      <c r="G110" s="4" t="inlineStr"/>
+      <c r="F110" s="6" t="n">
+        <v>1309</v>
+      </c>
+      <c r="G110" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1292→1309</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="n">
@@ -3216,8 +3846,14 @@
       <c r="E111" s="5" t="n">
         <v>1292</v>
       </c>
-      <c r="F111" s="6" t="n"/>
-      <c r="G111" s="4" t="inlineStr"/>
+      <c r="F111" s="6" t="n">
+        <v>1309</v>
+      </c>
+      <c r="G111" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1292→1309</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="n">
@@ -3241,8 +3877,14 @@
       <c r="E112" s="5" t="n">
         <v>1292</v>
       </c>
-      <c r="F112" s="6" t="n"/>
-      <c r="G112" s="4" t="inlineStr"/>
+      <c r="F112" s="6" t="n">
+        <v>1309</v>
+      </c>
+      <c r="G112" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1292→1309</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="n">
@@ -3266,8 +3908,14 @@
       <c r="E113" s="5" t="n">
         <v>1292</v>
       </c>
-      <c r="F113" s="6" t="n"/>
-      <c r="G113" s="4" t="inlineStr"/>
+      <c r="F113" s="6" t="n">
+        <v>1309</v>
+      </c>
+      <c r="G113" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1292→1309</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="n">
@@ -3291,8 +3939,14 @@
       <c r="E114" s="5" t="n">
         <v>2614</v>
       </c>
-      <c r="F114" s="6" t="n"/>
-      <c r="G114" s="4" t="inlineStr"/>
+      <c r="F114" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G114" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2614→1435</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="n">
@@ -3316,8 +3970,14 @@
       <c r="E115" s="5" t="n">
         <v>2614</v>
       </c>
-      <c r="F115" s="6" t="n"/>
-      <c r="G115" s="4" t="inlineStr"/>
+      <c r="F115" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G115" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2614→1435</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="n">
@@ -3341,8 +4001,14 @@
       <c r="E116" s="5" t="n">
         <v>2614</v>
       </c>
-      <c r="F116" s="6" t="n"/>
-      <c r="G116" s="4" t="inlineStr"/>
+      <c r="F116" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G116" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2614→1435</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="n">
@@ -3366,8 +4032,14 @@
       <c r="E117" s="5" t="n">
         <v>2614</v>
       </c>
-      <c r="F117" s="6" t="n"/>
-      <c r="G117" s="4" t="inlineStr"/>
+      <c r="F117" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G117" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2614→1435</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="n">
@@ -3391,8 +4063,14 @@
       <c r="E118" s="5" t="n">
         <v>2614</v>
       </c>
-      <c r="F118" s="6" t="n"/>
-      <c r="G118" s="4" t="inlineStr"/>
+      <c r="F118" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G118" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2614→1435</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="n">
@@ -3416,8 +4094,14 @@
       <c r="E119" s="5" t="n">
         <v>2614</v>
       </c>
-      <c r="F119" s="6" t="n"/>
-      <c r="G119" s="4" t="inlineStr"/>
+      <c r="F119" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G119" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2614→1435</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="n">
@@ -3441,8 +4125,14 @@
       <c r="E120" s="5" t="n">
         <v>2614</v>
       </c>
-      <c r="F120" s="6" t="n"/>
-      <c r="G120" s="4" t="inlineStr"/>
+      <c r="F120" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G120" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2614→1435</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="n">
@@ -3466,8 +4156,14 @@
       <c r="E121" s="5" t="n">
         <v>2658</v>
       </c>
-      <c r="F121" s="6" t="n"/>
-      <c r="G121" s="4" t="inlineStr"/>
+      <c r="F121" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G121" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2658→1435</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="n">
@@ -3491,8 +4187,14 @@
       <c r="E122" s="5" t="n">
         <v>2658</v>
       </c>
-      <c r="F122" s="6" t="n"/>
-      <c r="G122" s="4" t="inlineStr"/>
+      <c r="F122" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G122" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2658→1435</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="n">
@@ -3516,8 +4218,14 @@
       <c r="E123" s="5" t="n">
         <v>2658</v>
       </c>
-      <c r="F123" s="6" t="n"/>
-      <c r="G123" s="4" t="inlineStr"/>
+      <c r="F123" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G123" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2658→1435</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="n">
@@ -3541,8 +4249,14 @@
       <c r="E124" s="5" t="n">
         <v>2658</v>
       </c>
-      <c r="F124" s="6" t="n"/>
-      <c r="G124" s="4" t="inlineStr"/>
+      <c r="F124" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G124" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2658→1435</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="n">
@@ -3566,8 +4280,14 @@
       <c r="E125" s="5" t="n">
         <v>2658</v>
       </c>
-      <c r="F125" s="6" t="n"/>
-      <c r="G125" s="4" t="inlineStr"/>
+      <c r="F125" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G125" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2658→1435</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="n">
@@ -3591,8 +4311,14 @@
       <c r="E126" s="5" t="n">
         <v>2705</v>
       </c>
-      <c r="F126" s="6" t="n"/>
-      <c r="G126" s="4" t="inlineStr"/>
+      <c r="F126" s="6" t="n">
+        <v>1435</v>
+      </c>
+      <c r="G126" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2705→1435</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="n">
@@ -3616,8 +4342,14 @@
       <c r="E127" s="5" t="n">
         <v>856</v>
       </c>
-      <c r="F127" s="6" t="n"/>
-      <c r="G127" s="4" t="inlineStr"/>
+      <c r="F127" s="6" t="n">
+        <v>867</v>
+      </c>
+      <c r="G127" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  856→867</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="4" t="n">
@@ -3641,8 +4373,14 @@
       <c r="E128" s="5" t="n">
         <v>856</v>
       </c>
-      <c r="F128" s="6" t="n"/>
-      <c r="G128" s="4" t="inlineStr"/>
+      <c r="F128" s="6" t="n">
+        <v>867</v>
+      </c>
+      <c r="G128" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  856→867</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="n">
@@ -3666,8 +4404,14 @@
       <c r="E129" s="5" t="n">
         <v>1292</v>
       </c>
-      <c r="F129" s="6" t="n"/>
-      <c r="G129" s="4" t="inlineStr"/>
+      <c r="F129" s="6" t="n">
+        <v>1309</v>
+      </c>
+      <c r="G129" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1292→1309</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="n">
@@ -3691,8 +4435,14 @@
       <c r="E130" s="5" t="n">
         <v>1292</v>
       </c>
-      <c r="F130" s="6" t="n"/>
-      <c r="G130" s="4" t="inlineStr"/>
+      <c r="F130" s="6" t="n">
+        <v>1309</v>
+      </c>
+      <c r="G130" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1292→1309</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="n">
@@ -3716,8 +4466,14 @@
       <c r="E131" s="5" t="n">
         <v>1292</v>
       </c>
-      <c r="F131" s="6" t="n"/>
-      <c r="G131" s="4" t="inlineStr"/>
+      <c r="F131" s="6" t="n">
+        <v>1309</v>
+      </c>
+      <c r="G131" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1292→1309</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="n">
@@ -3741,8 +4497,14 @@
       <c r="E132" s="5" t="n">
         <v>1292</v>
       </c>
-      <c r="F132" s="6" t="n"/>
-      <c r="G132" s="4" t="inlineStr"/>
+      <c r="F132" s="6" t="n">
+        <v>1309</v>
+      </c>
+      <c r="G132" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1292→1309</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="n">
@@ -3766,8 +4528,14 @@
       <c r="E133" s="5" t="n">
         <v>906</v>
       </c>
-      <c r="F133" s="6" t="n"/>
-      <c r="G133" s="4" t="inlineStr"/>
+      <c r="F133" s="6" t="n">
+        <v>800</v>
+      </c>
+      <c r="G133" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  906→800</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="n">
@@ -3791,8 +4559,14 @@
       <c r="E134" s="5" t="n">
         <v>906</v>
       </c>
-      <c r="F134" s="6" t="n"/>
-      <c r="G134" s="4" t="inlineStr"/>
+      <c r="F134" s="6" t="n">
+        <v>800</v>
+      </c>
+      <c r="G134" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  906→800</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="n">
@@ -3816,8 +4590,14 @@
       <c r="E135" s="5" t="n">
         <v>906</v>
       </c>
-      <c r="F135" s="6" t="n"/>
-      <c r="G135" s="4" t="inlineStr"/>
+      <c r="F135" s="6" t="n">
+        <v>800</v>
+      </c>
+      <c r="G135" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  906→800</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="4" t="n">
@@ -3841,8 +4621,14 @@
       <c r="E136" s="5" t="n">
         <v>906</v>
       </c>
-      <c r="F136" s="6" t="n"/>
-      <c r="G136" s="4" t="inlineStr"/>
+      <c r="F136" s="6" t="n">
+        <v>800</v>
+      </c>
+      <c r="G136" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  906→800</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="n">
@@ -3866,8 +4652,14 @@
       <c r="E137" s="5" t="n">
         <v>906</v>
       </c>
-      <c r="F137" s="6" t="n"/>
-      <c r="G137" s="4" t="inlineStr"/>
+      <c r="F137" s="6" t="n">
+        <v>800</v>
+      </c>
+      <c r="G137" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  906→800</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="4" t="n">
@@ -3891,8 +4683,14 @@
       <c r="E138" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F138" s="6" t="n"/>
-      <c r="G138" s="4" t="inlineStr"/>
+      <c r="F138" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G138" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="n">
@@ -3916,8 +4714,14 @@
       <c r="E139" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F139" s="6" t="n"/>
-      <c r="G139" s="4" t="inlineStr"/>
+      <c r="F139" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G139" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="4" t="n">
@@ -3941,8 +4745,14 @@
       <c r="E140" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F140" s="6" t="n"/>
-      <c r="G140" s="4" t="inlineStr"/>
+      <c r="F140" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G140" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="n">
@@ -3966,8 +4776,14 @@
       <c r="E141" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F141" s="6" t="n"/>
-      <c r="G141" s="4" t="inlineStr"/>
+      <c r="F141" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G141" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="4" t="n">
@@ -3991,8 +4807,14 @@
       <c r="E142" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F142" s="6" t="n"/>
-      <c r="G142" s="4" t="inlineStr"/>
+      <c r="F142" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G142" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="n">
@@ -4016,8 +4838,14 @@
       <c r="E143" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F143" s="6" t="n"/>
-      <c r="G143" s="4" t="inlineStr"/>
+      <c r="F143" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G143" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="n">
@@ -4041,8 +4869,14 @@
       <c r="E144" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F144" s="6" t="n"/>
-      <c r="G144" s="4" t="inlineStr"/>
+      <c r="F144" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G144" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="n">
@@ -4066,8 +4900,14 @@
       <c r="E145" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F145" s="6" t="n"/>
-      <c r="G145" s="4" t="inlineStr"/>
+      <c r="F145" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G145" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="n">
@@ -4091,8 +4931,14 @@
       <c r="E146" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F146" s="6" t="n"/>
-      <c r="G146" s="4" t="inlineStr"/>
+      <c r="F146" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G146" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="n">
@@ -4116,8 +4962,14 @@
       <c r="E147" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F147" s="6" t="n"/>
-      <c r="G147" s="4" t="inlineStr"/>
+      <c r="F147" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G147" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="n">
@@ -4141,8 +4993,14 @@
       <c r="E148" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F148" s="6" t="n"/>
-      <c r="G148" s="4" t="inlineStr"/>
+      <c r="F148" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G148" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="n">
@@ -4166,8 +5024,14 @@
       <c r="E149" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F149" s="6" t="n"/>
-      <c r="G149" s="4" t="inlineStr"/>
+      <c r="F149" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G149" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="4" t="n">
@@ -4191,8 +5055,14 @@
       <c r="E150" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F150" s="6" t="n"/>
-      <c r="G150" s="4" t="inlineStr"/>
+      <c r="F150" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G150" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="n">
@@ -4216,8 +5086,14 @@
       <c r="E151" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F151" s="6" t="n"/>
-      <c r="G151" s="4" t="inlineStr"/>
+      <c r="F151" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G151" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="n">
@@ -4241,8 +5117,14 @@
       <c r="E152" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F152" s="6" t="n"/>
-      <c r="G152" s="4" t="inlineStr"/>
+      <c r="F152" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G152" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="n">
@@ -4266,8 +5148,14 @@
       <c r="E153" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F153" s="6" t="n"/>
-      <c r="G153" s="4" t="inlineStr"/>
+      <c r="F153" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G153" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="4" t="n">
@@ -4291,8 +5179,14 @@
       <c r="E154" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F154" s="6" t="n"/>
-      <c r="G154" s="4" t="inlineStr"/>
+      <c r="F154" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G154" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="n">
@@ -4316,8 +5210,14 @@
       <c r="E155" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F155" s="6" t="n"/>
-      <c r="G155" s="4" t="inlineStr"/>
+      <c r="F155" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G155" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="n">
@@ -4341,8 +5241,14 @@
       <c r="E156" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F156" s="6" t="n"/>
-      <c r="G156" s="4" t="inlineStr"/>
+      <c r="F156" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G156" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="n">
@@ -4366,8 +5272,14 @@
       <c r="E157" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F157" s="6" t="n"/>
-      <c r="G157" s="4" t="inlineStr"/>
+      <c r="F157" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G157" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="n">
@@ -4391,8 +5303,14 @@
       <c r="E158" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F158" s="6" t="n"/>
-      <c r="G158" s="4" t="inlineStr"/>
+      <c r="F158" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G158" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="n">
@@ -4416,8 +5334,14 @@
       <c r="E159" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F159" s="6" t="n"/>
-      <c r="G159" s="4" t="inlineStr"/>
+      <c r="F159" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G159" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="n">
@@ -4441,8 +5365,14 @@
       <c r="E160" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F160" s="6" t="n"/>
-      <c r="G160" s="4" t="inlineStr"/>
+      <c r="F160" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G160" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="n">
@@ -4466,8 +5396,14 @@
       <c r="E161" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F161" s="6" t="n"/>
-      <c r="G161" s="4" t="inlineStr"/>
+      <c r="F161" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G161" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="n">
@@ -4491,8 +5427,14 @@
       <c r="E162" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F162" s="6" t="n"/>
-      <c r="G162" s="4" t="inlineStr"/>
+      <c r="F162" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G162" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="n">
@@ -4516,8 +5458,14 @@
       <c r="E163" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F163" s="6" t="n"/>
-      <c r="G163" s="4" t="inlineStr"/>
+      <c r="F163" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G163" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="n">
@@ -4541,8 +5489,14 @@
       <c r="E164" s="5" t="n">
         <v>1392</v>
       </c>
-      <c r="F164" s="6" t="n"/>
-      <c r="G164" s="4" t="inlineStr"/>
+      <c r="F164" s="6" t="n">
+        <v>1434</v>
+      </c>
+      <c r="G164" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1392→1434</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="n">
@@ -4566,8 +5520,14 @@
       <c r="E165" s="5" t="n">
         <v>1853</v>
       </c>
-      <c r="F165" s="6" t="n"/>
-      <c r="G165" s="4" t="inlineStr"/>
+      <c r="F165" s="6" t="n">
+        <v>1780</v>
+      </c>
+      <c r="G165" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1853→1780</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="4" t="n">
@@ -4591,8 +5551,14 @@
       <c r="E166" s="5" t="n">
         <v>2216</v>
       </c>
-      <c r="F166" s="6" t="n"/>
-      <c r="G166" s="4" t="inlineStr"/>
+      <c r="F166" s="6" t="n">
+        <v>2048</v>
+      </c>
+      <c r="G166" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2216→2048</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="n">
@@ -4616,8 +5582,14 @@
       <c r="E167" s="5" t="n">
         <v>2216</v>
       </c>
-      <c r="F167" s="6" t="n"/>
-      <c r="G167" s="4" t="inlineStr"/>
+      <c r="F167" s="6" t="n">
+        <v>2048</v>
+      </c>
+      <c r="G167" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2216→2048</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="4" t="n">
@@ -4641,8 +5613,14 @@
       <c r="E168" s="5" t="n">
         <v>2216</v>
       </c>
-      <c r="F168" s="6" t="n"/>
-      <c r="G168" s="4" t="inlineStr"/>
+      <c r="F168" s="6" t="n">
+        <v>2048</v>
+      </c>
+      <c r="G168" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2216→2048</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="n">
@@ -4666,8 +5644,14 @@
       <c r="E169" s="5" t="n">
         <v>2216</v>
       </c>
-      <c r="F169" s="6" t="n"/>
-      <c r="G169" s="4" t="inlineStr"/>
+      <c r="F169" s="6" t="n">
+        <v>2048</v>
+      </c>
+      <c r="G169" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2216→2048</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="4" t="n">
@@ -4691,8 +5675,14 @@
       <c r="E170" s="5" t="n">
         <v>2384</v>
       </c>
-      <c r="F170" s="6" t="n"/>
-      <c r="G170" s="4" t="inlineStr"/>
+      <c r="F170" s="6" t="n">
+        <v>1910</v>
+      </c>
+      <c r="G170" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2384→1910</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="n">
@@ -4716,8 +5706,14 @@
       <c r="E171" s="5" t="n">
         <v>2384</v>
       </c>
-      <c r="F171" s="6" t="n"/>
-      <c r="G171" s="4" t="inlineStr"/>
+      <c r="F171" s="6" t="n">
+        <v>1910</v>
+      </c>
+      <c r="G171" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2384→1910</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="n">
@@ -4741,8 +5737,14 @@
       <c r="E172" s="5" t="n">
         <v>2384</v>
       </c>
-      <c r="F172" s="6" t="n"/>
-      <c r="G172" s="4" t="inlineStr"/>
+      <c r="F172" s="6" t="n">
+        <v>1910</v>
+      </c>
+      <c r="G172" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2384→1910</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="4" t="n">
@@ -4766,8 +5768,14 @@
       <c r="E173" s="5" t="n">
         <v>2384</v>
       </c>
-      <c r="F173" s="6" t="n"/>
-      <c r="G173" s="4" t="inlineStr"/>
+      <c r="F173" s="6" t="n">
+        <v>1910</v>
+      </c>
+      <c r="G173" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2384→1910</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="n">
@@ -4791,8 +5799,14 @@
       <c r="E174" s="5" t="n">
         <v>2359</v>
       </c>
-      <c r="F174" s="6" t="n"/>
-      <c r="G174" s="4" t="inlineStr"/>
+      <c r="F174" s="6" t="n">
+        <v>1910</v>
+      </c>
+      <c r="G174" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2359→1910</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="n">
@@ -4816,8 +5830,14 @@
       <c r="E175" s="5" t="n">
         <v>2359</v>
       </c>
-      <c r="F175" s="6" t="n"/>
-      <c r="G175" s="4" t="inlineStr"/>
+      <c r="F175" s="6" t="n">
+        <v>1910</v>
+      </c>
+      <c r="G175" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2359→1910</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="4" t="n">
@@ -4841,8 +5861,14 @@
       <c r="E176" s="5" t="n">
         <v>2359</v>
       </c>
-      <c r="F176" s="6" t="n"/>
-      <c r="G176" s="4" t="inlineStr"/>
+      <c r="F176" s="6" t="n">
+        <v>1910</v>
+      </c>
+      <c r="G176" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2359→1910</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="n">
@@ -4866,8 +5892,14 @@
       <c r="E177" s="5" t="n">
         <v>2359</v>
       </c>
-      <c r="F177" s="6" t="n"/>
-      <c r="G177" s="4" t="inlineStr"/>
+      <c r="F177" s="6" t="n">
+        <v>1910</v>
+      </c>
+      <c r="G177" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2359→1910</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="4" t="n">
@@ -4891,8 +5923,14 @@
       <c r="E178" s="5" t="n">
         <v>2256</v>
       </c>
-      <c r="F178" s="6" t="n"/>
-      <c r="G178" s="4" t="inlineStr"/>
+      <c r="F178" s="6" t="n">
+        <v>2119</v>
+      </c>
+      <c r="G178" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  2256→2119</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="n">
@@ -4916,8 +5954,14 @@
       <c r="E179" s="5" t="n">
         <v>2119</v>
       </c>
-      <c r="F179" s="6" t="n"/>
-      <c r="G179" s="4" t="inlineStr"/>
+      <c r="F179" s="6" t="n">
+        <v>2119</v>
+      </c>
+      <c r="G179" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致 なし</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="4" t="n">
@@ -4941,8 +5985,14 @@
       <c r="E180" s="5" t="n">
         <v>1147</v>
       </c>
-      <c r="F180" s="6" t="n"/>
-      <c r="G180" s="4" t="inlineStr"/>
+      <c r="F180" s="6" t="n">
+        <v>1017</v>
+      </c>
+      <c r="G180" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1147→1017</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="4" t="n">
@@ -4966,8 +6016,14 @@
       <c r="E181" s="5" t="n">
         <v>1147</v>
       </c>
-      <c r="F181" s="6" t="n"/>
-      <c r="G181" s="4" t="inlineStr"/>
+      <c r="F181" s="6" t="n">
+        <v>1017</v>
+      </c>
+      <c r="G181" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1147→1017</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="4" t="n">
@@ -4991,8 +6047,14 @@
       <c r="E182" s="5" t="n">
         <v>1147</v>
       </c>
-      <c r="F182" s="6" t="n"/>
-      <c r="G182" s="4" t="inlineStr"/>
+      <c r="F182" s="6" t="n">
+        <v>1017</v>
+      </c>
+      <c r="G182" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1147→1017</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="4" t="n">
@@ -5016,8 +6078,14 @@
       <c r="E183" s="5" t="n">
         <v>1147</v>
       </c>
-      <c r="F183" s="6" t="n"/>
-      <c r="G183" s="4" t="inlineStr"/>
+      <c r="F183" s="6" t="n">
+        <v>1017</v>
+      </c>
+      <c r="G183" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1147→1017</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="4" t="n">
@@ -5041,8 +6109,14 @@
       <c r="E184" s="5" t="n">
         <v>1147</v>
       </c>
-      <c r="F184" s="6" t="n"/>
-      <c r="G184" s="4" t="inlineStr"/>
+      <c r="F184" s="6" t="n">
+        <v>1017</v>
+      </c>
+      <c r="G184" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1147→1017</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="4" t="n">
@@ -5066,8 +6140,14 @@
       <c r="E185" s="5" t="n">
         <v>1147</v>
       </c>
-      <c r="F185" s="6" t="n"/>
-      <c r="G185" s="4" t="inlineStr"/>
+      <c r="F185" s="6" t="n">
+        <v>1017</v>
+      </c>
+      <c r="G185" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1147→1017</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="4" t="n">
@@ -5091,8 +6171,14 @@
       <c r="E186" s="5" t="n">
         <v>1147</v>
       </c>
-      <c r="F186" s="6" t="n"/>
-      <c r="G186" s="4" t="inlineStr"/>
+      <c r="F186" s="6" t="n">
+        <v>1017</v>
+      </c>
+      <c r="G186" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1147→1017</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="n">
@@ -5116,8 +6202,14 @@
       <c r="E187" s="5" t="n">
         <v>1147</v>
       </c>
-      <c r="F187" s="6" t="n"/>
-      <c r="G187" s="4" t="inlineStr"/>
+      <c r="F187" s="6" t="n">
+        <v>1017</v>
+      </c>
+      <c r="G187" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1147→1017</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="4" t="n">
@@ -5141,8 +6233,14 @@
       <c r="E188" s="5" t="n">
         <v>1147</v>
       </c>
-      <c r="F188" s="6" t="n"/>
-      <c r="G188" s="4" t="inlineStr"/>
+      <c r="F188" s="6" t="n">
+        <v>1017</v>
+      </c>
+      <c r="G188" s="4" t="inlineStr">
+        <is>
+          <t>✅更新済・実測一致  1147→1017</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="7" t="n">
@@ -5167,7 +6265,11 @@
         <v>989</v>
       </c>
       <c r="F189" s="6" t="n"/>
-      <c r="G189" s="7" t="inlineStr"/>
+      <c r="G189" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="7" t="n">
@@ -5192,7 +6294,11 @@
         <v>989</v>
       </c>
       <c r="F190" s="6" t="n"/>
-      <c r="G190" s="7" t="inlineStr"/>
+      <c r="G190" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="7" t="n">
@@ -5217,7 +6323,11 @@
         <v>989</v>
       </c>
       <c r="F191" s="6" t="n"/>
-      <c r="G191" s="7" t="inlineStr"/>
+      <c r="G191" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="7" t="n">
@@ -5242,7 +6352,11 @@
         <v>989</v>
       </c>
       <c r="F192" s="6" t="n"/>
-      <c r="G192" s="7" t="inlineStr"/>
+      <c r="G192" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="7" t="n">
@@ -5267,7 +6381,11 @@
         <v>2636</v>
       </c>
       <c r="F193" s="6" t="n"/>
-      <c r="G193" s="7" t="inlineStr"/>
+      <c r="G193" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="7" t="n">
@@ -5292,7 +6410,11 @@
         <v>3952</v>
       </c>
       <c r="F194" s="6" t="n"/>
-      <c r="G194" s="7" t="inlineStr"/>
+      <c r="G194" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="7" t="n">
@@ -5317,7 +6439,11 @@
         <v>2636</v>
       </c>
       <c r="F195" s="6" t="n"/>
-      <c r="G195" s="7" t="inlineStr"/>
+      <c r="G195" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="7" t="n">
@@ -5342,7 +6468,11 @@
         <v>2527</v>
       </c>
       <c r="F196" s="6" t="n"/>
-      <c r="G196" s="7" t="inlineStr"/>
+      <c r="G196" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="7" t="n">
@@ -5367,7 +6497,11 @@
         <v>2527</v>
       </c>
       <c r="F197" s="6" t="n"/>
-      <c r="G197" s="7" t="inlineStr"/>
+      <c r="G197" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="7" t="n">
@@ -5392,7 +6526,11 @@
         <v>2527</v>
       </c>
       <c r="F198" s="6" t="n"/>
-      <c r="G198" s="7" t="inlineStr"/>
+      <c r="G198" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="7" t="n">
@@ -5417,7 +6555,11 @@
         <v>2527</v>
       </c>
       <c r="F199" s="6" t="n"/>
-      <c r="G199" s="7" t="inlineStr"/>
+      <c r="G199" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="7" t="n">
@@ -5442,7 +6584,11 @@
         <v>2527</v>
       </c>
       <c r="F200" s="6" t="n"/>
-      <c r="G200" s="7" t="inlineStr"/>
+      <c r="G200" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="7" t="n">
@@ -5467,7 +6613,11 @@
         <v>2527</v>
       </c>
       <c r="F201" s="6" t="n"/>
-      <c r="G201" s="7" t="inlineStr"/>
+      <c r="G201" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="7" t="n">
@@ -5492,7 +6642,11 @@
         <v>2636</v>
       </c>
       <c r="F202" s="6" t="n"/>
-      <c r="G202" s="7" t="inlineStr"/>
+      <c r="G202" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="7" t="n">
@@ -5517,7 +6671,11 @@
         <v>2636</v>
       </c>
       <c r="F203" s="6" t="n"/>
-      <c r="G203" s="7" t="inlineStr"/>
+      <c r="G203" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="7" t="n">
@@ -5542,7 +6700,11 @@
         <v>3952</v>
       </c>
       <c r="F204" s="6" t="n"/>
-      <c r="G204" s="7" t="inlineStr"/>
+      <c r="G204" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="7" t="n">
@@ -5567,7 +6729,11 @@
         <v>3952</v>
       </c>
       <c r="F205" s="6" t="n"/>
-      <c r="G205" s="7" t="inlineStr"/>
+      <c r="G205" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="7" t="n">
@@ -5592,7 +6758,11 @@
         <v>831</v>
       </c>
       <c r="F206" s="6" t="n"/>
-      <c r="G206" s="7" t="inlineStr"/>
+      <c r="G206" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="7" t="n">
@@ -5617,7 +6787,11 @@
         <v>729</v>
       </c>
       <c r="F207" s="6" t="n"/>
-      <c r="G207" s="7" t="inlineStr"/>
+      <c r="G207" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="7" t="n">
@@ -5642,7 +6816,11 @@
         <v>729</v>
       </c>
       <c r="F208" s="6" t="n"/>
-      <c r="G208" s="7" t="inlineStr"/>
+      <c r="G208" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="7" t="n">
@@ -5667,7 +6845,11 @@
         <v>729</v>
       </c>
       <c r="F209" s="6" t="n"/>
-      <c r="G209" s="7" t="inlineStr"/>
+      <c r="G209" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="7" t="n">
@@ -5692,7 +6874,11 @@
         <v>729</v>
       </c>
       <c r="F210" s="6" t="n"/>
-      <c r="G210" s="7" t="inlineStr"/>
+      <c r="G210" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="7" t="n">
@@ -5717,7 +6903,11 @@
         <v>729</v>
       </c>
       <c r="F211" s="6" t="n"/>
-      <c r="G211" s="7" t="inlineStr"/>
+      <c r="G211" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="7" t="n">
@@ -5742,7 +6932,11 @@
         <v>2731</v>
       </c>
       <c r="F212" s="6" t="n"/>
-      <c r="G212" s="7" t="inlineStr"/>
+      <c r="G212" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="7" t="n">
@@ -5767,7 +6961,11 @@
         <v>2731</v>
       </c>
       <c r="F213" s="6" t="n"/>
-      <c r="G213" s="7" t="inlineStr"/>
+      <c r="G213" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="7" t="n">
@@ -5792,7 +6990,11 @@
         <v>2731</v>
       </c>
       <c r="F214" s="6" t="n"/>
-      <c r="G214" s="7" t="inlineStr"/>
+      <c r="G214" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="7" t="n">
@@ -5817,7 +7019,11 @@
         <v>2731</v>
       </c>
       <c r="F215" s="6" t="n"/>
-      <c r="G215" s="7" t="inlineStr"/>
+      <c r="G215" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="7" t="n">
@@ -5842,7 +7048,11 @@
         <v>2731</v>
       </c>
       <c r="F216" s="6" t="n"/>
-      <c r="G216" s="7" t="inlineStr"/>
+      <c r="G216" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="7" t="n">
@@ -5867,7 +7077,11 @@
         <v>2731</v>
       </c>
       <c r="F217" s="6" t="n"/>
-      <c r="G217" s="7" t="inlineStr"/>
+      <c r="G217" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="7" t="n">
@@ -5892,7 +7106,11 @@
         <v>2731</v>
       </c>
       <c r="F218" s="6" t="n"/>
-      <c r="G218" s="7" t="inlineStr"/>
+      <c r="G218" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="7" t="n">
@@ -5917,7 +7135,11 @@
         <v>2731</v>
       </c>
       <c r="F219" s="6" t="n"/>
-      <c r="G219" s="7" t="inlineStr"/>
+      <c r="G219" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="7" t="n">
@@ -5942,7 +7164,11 @@
         <v>2731</v>
       </c>
       <c r="F220" s="6" t="n"/>
-      <c r="G220" s="7" t="inlineStr"/>
+      <c r="G220" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="7" t="n">
@@ -5967,7 +7193,11 @@
         <v>1967</v>
       </c>
       <c r="F221" s="6" t="n"/>
-      <c r="G221" s="7" t="inlineStr"/>
+      <c r="G221" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="7" t="n">
@@ -5992,7 +7222,11 @@
         <v>1967</v>
       </c>
       <c r="F222" s="6" t="n"/>
-      <c r="G222" s="7" t="inlineStr"/>
+      <c r="G222" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="7" t="n">
@@ -6017,7 +7251,11 @@
         <v>1967</v>
       </c>
       <c r="F223" s="6" t="n"/>
-      <c r="G223" s="7" t="inlineStr"/>
+      <c r="G223" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="7" t="n">
@@ -6042,7 +7280,11 @@
         <v>1711</v>
       </c>
       <c r="F224" s="6" t="n"/>
-      <c r="G224" s="7" t="inlineStr"/>
+      <c r="G224" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="7" t="n">
@@ -6067,7 +7309,11 @@
         <v>1711</v>
       </c>
       <c r="F225" s="6" t="n"/>
-      <c r="G225" s="7" t="inlineStr"/>
+      <c r="G225" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="7" t="n">
@@ -6092,7 +7338,11 @@
         <v>1711</v>
       </c>
       <c r="F226" s="6" t="n"/>
-      <c r="G226" s="7" t="inlineStr"/>
+      <c r="G226" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="7" t="n">
@@ -6117,7 +7367,11 @@
         <v>3256</v>
       </c>
       <c r="F227" s="6" t="n"/>
-      <c r="G227" s="7" t="inlineStr"/>
+      <c r="G227" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="7" t="n">
@@ -6142,7 +7396,11 @@
         <v>3256</v>
       </c>
       <c r="F228" s="6" t="n"/>
-      <c r="G228" s="7" t="inlineStr"/>
+      <c r="G228" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="7" t="n">
@@ -6167,7 +7425,11 @@
         <v>3518</v>
       </c>
       <c r="F229" s="6" t="n"/>
-      <c r="G229" s="7" t="inlineStr"/>
+      <c r="G229" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="7" t="n">
@@ -6192,7 +7454,11 @@
         <v>3518</v>
       </c>
       <c r="F230" s="6" t="n"/>
-      <c r="G230" s="7" t="inlineStr"/>
+      <c r="G230" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="7" t="n">
@@ -6217,7 +7483,7 @@
       <c r="F231" s="6" t="n"/>
       <c r="G231" s="7" t="inlineStr">
         <is>
-          <t>原価未登録</t>
+          <t>対象外(非ACTIVE)</t>
         </is>
       </c>
     </row>
@@ -6244,7 +7510,11 @@
         <v>2072</v>
       </c>
       <c r="F232" s="6" t="n"/>
-      <c r="G232" s="7" t="inlineStr"/>
+      <c r="G232" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="7" t="n">
@@ -6269,7 +7539,11 @@
         <v>2072</v>
       </c>
       <c r="F233" s="6" t="n"/>
-      <c r="G233" s="7" t="inlineStr"/>
+      <c r="G233" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="7" t="n">
@@ -6294,7 +7568,11 @@
         <v>2072</v>
       </c>
       <c r="F234" s="6" t="n"/>
-      <c r="G234" s="7" t="inlineStr"/>
+      <c r="G234" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="7" t="n">
@@ -6319,7 +7597,11 @@
         <v>2492</v>
       </c>
       <c r="F235" s="6" t="n"/>
-      <c r="G235" s="7" t="inlineStr"/>
+      <c r="G235" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="7" t="n">
@@ -6344,7 +7626,11 @@
         <v>5339</v>
       </c>
       <c r="F236" s="6" t="n"/>
-      <c r="G236" s="7" t="inlineStr"/>
+      <c r="G236" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="7" t="n">
@@ -6369,7 +7655,11 @@
         <v>5339</v>
       </c>
       <c r="F237" s="6" t="n"/>
-      <c r="G237" s="7" t="inlineStr"/>
+      <c r="G237" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="7" t="n">
@@ -6394,7 +7684,11 @@
         <v>5339</v>
       </c>
       <c r="F238" s="6" t="n"/>
-      <c r="G238" s="7" t="inlineStr"/>
+      <c r="G238" s="7" t="inlineStr">
+        <is>
+          <t>対象外(非ACTIVE)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>